<commit_message>
semana 9 de 2026 envio de IRAs
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/revision_IRAExt_semanal.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/revision_IRAExt_semanal.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -410,6 +410,11 @@
           <t>8</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -451,6 +456,9 @@
       <c r="K2">
         <v>32</v>
       </c>
+      <c r="L2">
+        <v>31</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -483,6 +491,9 @@
       <c r="K3">
         <v>82</v>
       </c>
+      <c r="L3">
+        <v>168</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -550,6 +561,9 @@
       <c r="K5">
         <v>2</v>
       </c>
+      <c r="L5">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -591,6 +605,9 @@
       <c r="K6">
         <v>86</v>
       </c>
+      <c r="L6">
+        <v>966</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -632,6 +649,9 @@
       <c r="K7">
         <v>34</v>
       </c>
+      <c r="L7">
+        <v>39</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -673,6 +693,9 @@
       <c r="K8">
         <v>32</v>
       </c>
+      <c r="L8">
+        <v>39</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -714,6 +737,9 @@
       <c r="K9">
         <v>1</v>
       </c>
+      <c r="L9">
+        <v>2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -784,6 +810,9 @@
       <c r="K11">
         <v>1</v>
       </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -810,6 +839,9 @@
       <c r="K12">
         <v>3</v>
       </c>
+      <c r="L12">
+        <v>2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -845,6 +877,9 @@
       <c r="K13">
         <v>6</v>
       </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -883,6 +918,9 @@
       <c r="K14">
         <v>1</v>
       </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -915,6 +953,9 @@
       <c r="K15">
         <v>2</v>
       </c>
+      <c r="L15">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -967,6 +1008,9 @@
       <c r="K17">
         <v>2</v>
       </c>
+      <c r="L17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1060,6 +1104,9 @@
       <c r="K20">
         <v>6</v>
       </c>
+      <c r="L20">
+        <v>6</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1101,6 +1148,9 @@
       <c r="K21">
         <v>45</v>
       </c>
+      <c r="L21">
+        <v>60</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1153,6 +1203,9 @@
       <c r="K23">
         <v>2</v>
       </c>
+      <c r="L23">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1194,6 +1247,9 @@
       <c r="K24">
         <v>214</v>
       </c>
+      <c r="L24">
+        <v>442</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1214,6 +1270,9 @@
       <c r="K25">
         <v>0</v>
       </c>
+      <c r="L25">
+        <v>594</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1255,6 +1314,9 @@
       <c r="K26">
         <v>0</v>
       </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1293,6 +1355,12 @@
       <c r="J27">
         <v>94</v>
       </c>
+      <c r="K27">
+        <v>66</v>
+      </c>
+      <c r="L27">
+        <v>51</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1334,6 +1402,9 @@
       <c r="K28">
         <v>3</v>
       </c>
+      <c r="L28">
+        <v>12</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1375,6 +1446,9 @@
       <c r="K29">
         <v>43</v>
       </c>
+      <c r="L29">
+        <v>71</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1416,6 +1490,9 @@
       <c r="K30">
         <v>42</v>
       </c>
+      <c r="L30">
+        <v>56</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1457,6 +1534,9 @@
       <c r="K31">
         <v>11</v>
       </c>
+      <c r="L31">
+        <v>13</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1498,95 +1578,83 @@
       <c r="K32">
         <v>110</v>
       </c>
+      <c r="L32">
+        <v>51</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6600102402</t>
+          <t>6600102288</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>IPS CENTRO DE MEDICINA INTEGRATIVA SAS</t>
-        </is>
-      </c>
-      <c r="G33">
-        <v>2</v>
+          <t>SALUD PYP SAS</t>
+        </is>
+      </c>
+      <c r="K33">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6600102411</t>
+          <t>6600102402</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>03</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SERVICIOS DE SALUD IPS SURAMERICANA SA</t>
-        </is>
-      </c>
-      <c r="F34">
-        <v>5</v>
-      </c>
-      <c r="H34">
-        <v>9</v>
-      </c>
-      <c r="I34">
-        <v>11</v>
-      </c>
-      <c r="J34">
-        <v>18</v>
+          <t>IPS CENTRO DE MEDICINA INTEGRATIVA SAS</t>
+        </is>
+      </c>
+      <c r="G34">
+        <v>2</v>
+      </c>
+      <c r="L34">
+        <v>12</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6600102446</t>
+          <t>6600102411</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CAJA COLOMBIANA DE SUBSIDIO FAMILIAR COLSUBSIDIO</t>
-        </is>
-      </c>
-      <c r="D35">
-        <v>108</v>
-      </c>
-      <c r="E35">
-        <v>61</v>
+          <t>SERVICIOS DE SALUD IPS SURAMERICANA SA</t>
+        </is>
       </c>
       <c r="F35">
-        <v>123</v>
-      </c>
-      <c r="G35">
-        <v>67</v>
+        <v>5</v>
       </c>
       <c r="H35">
-        <v>99</v>
+        <v>9</v>
       </c>
       <c r="I35">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="J35">
-        <v>97</v>
-      </c>
-      <c r="K35">
-        <v>98</v>
+        <v>18</v>
+      </c>
+      <c r="L35">
+        <v>14</v>
       </c>
     </row>
     <row r="36">
@@ -1597,7 +1665,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>02</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1606,34 +1674,37 @@
         </is>
       </c>
       <c r="D36">
-        <v>65</v>
+        <v>108</v>
       </c>
       <c r="E36">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F36">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="G36">
-        <v>42</v>
+        <v>67</v>
       </c>
       <c r="H36">
-        <v>48</v>
+        <v>99</v>
       </c>
       <c r="I36">
-        <v>39</v>
+        <v>71</v>
       </c>
       <c r="J36">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="K36">
-        <v>57</v>
+        <v>98</v>
+      </c>
+      <c r="L36">
+        <v>20</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6600102453</t>
+          <t>6600102446</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1643,79 +1714,85 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>VITALCARE IPS SAS</t>
+          <t>CAJA COLOMBIANA DE SUBSIDIO FAMILIAR COLSUBSIDIO</t>
         </is>
       </c>
       <c r="D37">
-        <v>13</v>
+        <v>65</v>
       </c>
       <c r="E37">
-        <v>8</v>
+        <v>57</v>
       </c>
       <c r="F37">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G37">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="H37">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="I37">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="J37">
-        <v>14</v>
+        <v>44</v>
       </c>
       <c r="K37">
-        <v>29</v>
+        <v>57</v>
+      </c>
+      <c r="L37">
+        <v>112</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>6600102477</t>
+          <t>6600102453</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>02</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>EMPRESA DE MEDICINA INTEGRAL EMI SA - SERVICIO DE</t>
+          <t>VITALCARE IPS SAS</t>
         </is>
       </c>
       <c r="D38">
-        <v>210</v>
+        <v>13</v>
       </c>
       <c r="E38">
-        <v>190</v>
+        <v>8</v>
       </c>
       <c r="F38">
-        <v>169</v>
+        <v>15</v>
       </c>
       <c r="G38">
-        <v>168</v>
+        <v>10</v>
       </c>
       <c r="H38">
-        <v>172</v>
+        <v>8</v>
       </c>
       <c r="I38">
-        <v>173</v>
+        <v>19</v>
       </c>
       <c r="J38">
-        <v>166</v>
+        <v>14</v>
       </c>
       <c r="K38">
-        <v>182</v>
+        <v>29</v>
+      </c>
+      <c r="L38">
+        <v>11</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>6600102601</t>
+          <t>6600102477</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1725,32 +1802,35 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>VIRREY SOLIS SA PINARES</t>
+          <t>EMPRESA DE MEDICINA INTEGRAL EMI SA - SERVICIO DE</t>
         </is>
       </c>
       <c r="D39">
-        <v>84</v>
+        <v>210</v>
       </c>
       <c r="E39">
-        <v>83</v>
+        <v>190</v>
       </c>
       <c r="F39">
-        <v>128</v>
+        <v>169</v>
       </c>
       <c r="G39">
-        <v>54</v>
+        <v>168</v>
       </c>
       <c r="H39">
-        <v>93</v>
+        <v>172</v>
       </c>
       <c r="I39">
-        <v>90</v>
+        <v>173</v>
       </c>
       <c r="J39">
-        <v>98</v>
+        <v>166</v>
       </c>
       <c r="K39">
-        <v>59</v>
+        <v>182</v>
+      </c>
+      <c r="L39">
+        <v>194</v>
       </c>
     </row>
     <row r="40">
@@ -1761,37 +1841,40 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>03</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>VIRREY SOLIS IPS LAGO</t>
+          <t>VIRREY SOLIS SA PINARES</t>
         </is>
       </c>
       <c r="D40">
-        <v>154</v>
+        <v>84</v>
       </c>
       <c r="E40">
-        <v>151</v>
+        <v>83</v>
       </c>
       <c r="F40">
-        <v>188</v>
+        <v>128</v>
       </c>
       <c r="G40">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="H40">
-        <v>127</v>
+        <v>93</v>
       </c>
       <c r="I40">
-        <v>134</v>
+        <v>90</v>
       </c>
       <c r="J40">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="K40">
-        <v>165</v>
+        <v>59</v>
+      </c>
+      <c r="L40">
+        <v>63</v>
       </c>
     </row>
     <row r="41">
@@ -1802,37 +1885,40 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>06</t>
+          <t>03</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>VIRREY SOLIS IPS SA ALPES</t>
+          <t>VIRREY SOLIS IPS LAGO</t>
         </is>
       </c>
       <c r="D41">
-        <v>9</v>
+        <v>154</v>
       </c>
       <c r="E41">
-        <v>9</v>
+        <v>151</v>
       </c>
       <c r="F41">
-        <v>3</v>
+        <v>188</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="H41">
-        <v>4</v>
+        <v>127</v>
       </c>
       <c r="I41">
-        <v>2</v>
+        <v>134</v>
       </c>
       <c r="J41">
-        <v>5</v>
+        <v>147</v>
       </c>
       <c r="K41">
-        <v>3</v>
+        <v>165</v>
+      </c>
+      <c r="L41">
+        <v>151</v>
       </c>
     </row>
     <row r="42">
@@ -1843,37 +1929,40 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>06</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>VIRREY SOLIS IPS SA LA REBECA</t>
+          <t>VIRREY SOLIS IPS SA ALPES</t>
         </is>
       </c>
       <c r="D42">
-        <v>89</v>
+        <v>9</v>
       </c>
       <c r="E42">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="F42">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="G42">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="H42">
-        <v>119</v>
+        <v>4</v>
       </c>
       <c r="I42">
-        <v>77</v>
+        <v>2</v>
       </c>
       <c r="J42">
-        <v>87</v>
+        <v>5</v>
       </c>
       <c r="K42">
-        <v>115</v>
+        <v>3</v>
+      </c>
+      <c r="L42">
+        <v>48</v>
       </c>
     </row>
     <row r="43">
@@ -1884,69 +1973,75 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08</t>
+          <t>07</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>VIRREY SOLIS IPS SA CERRITOS</t>
-        </is>
+          <t>VIRREY SOLIS IPS SA LA REBECA</t>
+        </is>
+      </c>
+      <c r="D43">
+        <v>89</v>
+      </c>
+      <c r="E43">
+        <v>93</v>
+      </c>
+      <c r="F43">
+        <v>95</v>
+      </c>
+      <c r="G43">
+        <v>44</v>
+      </c>
+      <c r="H43">
+        <v>119</v>
       </c>
       <c r="I43">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="J43">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="K43">
-        <v>18</v>
+        <v>115</v>
+      </c>
+      <c r="L43">
+        <v>90</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>6600102793</t>
+          <t>6600102601</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>08</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CENTRO MEDICO PEREIRA COLSANITAS</t>
-        </is>
-      </c>
-      <c r="D44">
-        <v>1</v>
-      </c>
-      <c r="E44">
-        <v>2</v>
-      </c>
-      <c r="F44">
-        <v>3</v>
-      </c>
-      <c r="G44">
-        <v>2</v>
-      </c>
-      <c r="H44">
-        <v>6</v>
+          <t>VIRREY SOLIS IPS SA CERRITOS</t>
+        </is>
       </c>
       <c r="I44">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="J44">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="K44">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="L44">
+        <v>88</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>6600102893</t>
+          <t>6600102793</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1956,38 +2051,41 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>NEUROMEDICA SAS</t>
+          <t>CENTRO MEDICO PEREIRA COLSANITAS</t>
         </is>
       </c>
       <c r="D45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G45">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J45">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K45">
-        <v>0</v>
+        <v>2</v>
+      </c>
+      <c r="L45">
+        <v>5</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>6600103012</t>
+          <t>6600102893</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1997,35 +2095,41 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SPORT MEDICAL IPS GUSTAVO PORTELA SAS</t>
+          <t>NEUROMEDICA SAS</t>
         </is>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="E46">
-        <v>24</v>
+        <v>0</v>
+      </c>
+      <c r="F46">
+        <v>0</v>
       </c>
       <c r="G46">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="I46">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="J46">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K46">
-        <v>7</v>
+        <v>0</v>
+      </c>
+      <c r="L46">
+        <v>0</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>6600103078</t>
+          <t>6600103012</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2035,38 +2139,38 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COOMEVA EXPERIENCIA MEDICA SAS</t>
+          <t>SPORT MEDICAL IPS GUSTAVO PORTELA SAS</t>
         </is>
       </c>
       <c r="D47">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E47">
-        <v>4</v>
-      </c>
-      <c r="F47">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="G47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H47">
+        <v>7</v>
+      </c>
+      <c r="I47">
+        <v>20</v>
+      </c>
+      <c r="J47">
+        <v>8</v>
+      </c>
+      <c r="K47">
+        <v>7</v>
+      </c>
+      <c r="L47">
         <v>6</v>
-      </c>
-      <c r="I47">
-        <v>2</v>
-      </c>
-      <c r="J47">
-        <v>3</v>
-      </c>
-      <c r="K47">
-        <v>4</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>6600103144</t>
+          <t>6600103078</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2076,38 +2180,41 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>CLINICA LOS NEVADOS SAS</t>
+          <t>COOMEVA EXPERIENCIA MEDICA SAS</t>
         </is>
       </c>
       <c r="D48">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E48">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F48">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G48">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H48">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I48">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J48">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K48">
-        <v>0</v>
+        <v>4</v>
+      </c>
+      <c r="L48">
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>6600103334</t>
+          <t>6600103144</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2117,35 +2224,41 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>CLINICA CENTRAL DEL EJE SAS</t>
+          <t>CLINICA LOS NEVADOS SAS</t>
         </is>
       </c>
       <c r="D49">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G49">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H49">
+        <v>0</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49">
+        <v>2</v>
+      </c>
+      <c r="K49">
+        <v>0</v>
+      </c>
+      <c r="L49">
         <v>3</v>
-      </c>
-      <c r="I49">
-        <v>0</v>
-      </c>
-      <c r="K49">
-        <v>6</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>6600103414</t>
+          <t>6600103334</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2155,155 +2268,208 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>CLINICA MEDICA TURIN SAS</t>
+          <t>CLINICA CENTRAL DEL EJE SAS</t>
         </is>
       </c>
       <c r="D50">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E50">
         <v>0</v>
       </c>
       <c r="F50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G50">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I50">
         <v>0</v>
       </c>
-      <c r="J50">
-        <v>0</v>
-      </c>
       <c r="K50">
-        <v>0</v>
+        <v>6</v>
+      </c>
+      <c r="L50">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>6600161600</t>
+          <t>6600103414</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>01</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>EPMSC PEREIRA</t>
+          <t>CLINICA MEDICA TURIN SAS</t>
         </is>
       </c>
       <c r="D51">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E51">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G51">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="H51">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I51">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J51">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K51">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="L51">
+        <v>0</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>6600171151</t>
+          <t>6600161600</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>99</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>SANIDAD POLICIA NACIONAL RISARALDA</t>
+          <t>EPMSC PEREIRA</t>
         </is>
       </c>
       <c r="D52">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E52">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="F52">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G52">
         <v>16</v>
       </c>
       <c r="H52">
-        <v>88</v>
+        <v>10</v>
       </c>
       <c r="I52">
-        <v>316</v>
+        <v>4</v>
       </c>
       <c r="J52">
         <v>9</v>
       </c>
       <c r="K52">
-        <v>13</v>
+        <v>5</v>
+      </c>
+      <c r="L52">
+        <v>9</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>6600171151</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>SANIDAD POLICIA NACIONAL RISARALDA</t>
+        </is>
+      </c>
+      <c r="D53">
+        <v>10</v>
+      </c>
+      <c r="E53">
+        <v>29</v>
+      </c>
+      <c r="F53">
+        <v>11</v>
+      </c>
+      <c r="G53">
+        <v>16</v>
+      </c>
+      <c r="H53">
+        <v>88</v>
+      </c>
+      <c r="I53">
+        <v>316</v>
+      </c>
+      <c r="J53">
+        <v>9</v>
+      </c>
+      <c r="K53">
+        <v>13</v>
+      </c>
+      <c r="L53">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>6600183029</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>BATALLON SAN MATEO</t>
         </is>
       </c>
-      <c r="D53">
+      <c r="D54">
         <v>7</v>
       </c>
-      <c r="E53">
+      <c r="E54">
         <v>11</v>
       </c>
-      <c r="F53">
+      <c r="F54">
         <v>13</v>
       </c>
-      <c r="G53">
+      <c r="G54">
         <v>19</v>
       </c>
-      <c r="H53">
+      <c r="H54">
         <v>25</v>
       </c>
-      <c r="I53">
+      <c r="I54">
         <v>26</v>
       </c>
-      <c r="J53">
+      <c r="J54">
         <v>43</v>
       </c>
-      <c r="K53">
+      <c r="K54">
         <v>54</v>
+      </c>
+      <c r="L54">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
envio de IRA semana 14 2026
</commit_message>
<xml_diff>
--- a/Boletin_ Epi_Pereira/Datos/revision_IRAExt_semanal.xlsx
+++ b/Boletin_ Epi_Pereira/Datos/revision_IRAExt_semanal.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:Q57"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -435,6 +435,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -508,6 +513,9 @@
       <c r="P3">
         <v>28</v>
       </c>
+      <c r="Q3">
+        <v>30</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -561,6 +569,9 @@
       <c r="O4">
         <v>69</v>
       </c>
+      <c r="Q4">
+        <v>46</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -649,6 +660,9 @@
       <c r="P6">
         <v>4</v>
       </c>
+      <c r="Q6">
+        <v>2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -705,6 +719,9 @@
       <c r="P7">
         <v>77</v>
       </c>
+      <c r="Q7">
+        <v>34</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -761,6 +778,9 @@
       <c r="P8">
         <v>31</v>
       </c>
+      <c r="Q8">
+        <v>26</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -817,6 +837,9 @@
       <c r="P9">
         <v>24</v>
       </c>
+      <c r="Q9">
+        <v>13</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -911,6 +934,9 @@
       <c r="L11">
         <v>1</v>
       </c>
+      <c r="Q11">
+        <v>2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -949,6 +975,9 @@
       <c r="P12">
         <v>1</v>
       </c>
+      <c r="Q12">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1028,6 +1057,9 @@
       <c r="P14">
         <v>1</v>
       </c>
+      <c r="Q14">
+        <v>4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1078,6 +1110,9 @@
       <c r="O15">
         <v>4</v>
       </c>
+      <c r="Q15">
+        <v>2</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1122,6 +1157,9 @@
       <c r="O16">
         <v>2</v>
       </c>
+      <c r="Q16">
+        <v>1</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1145,6 +1183,9 @@
       <c r="N17">
         <v>1</v>
       </c>
+      <c r="Q17">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1232,6 +1273,9 @@
       <c r="P20">
         <v>1</v>
       </c>
+      <c r="Q20">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1317,6 +1361,9 @@
       <c r="O22">
         <v>2</v>
       </c>
+      <c r="Q22">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1393,6 +1440,9 @@
       <c r="P24">
         <v>36</v>
       </c>
+      <c r="Q24">
+        <v>35</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1457,6 +1507,9 @@
       <c r="O26">
         <v>1</v>
       </c>
+      <c r="Q26">
+        <v>1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1495,6 +1548,9 @@
       <c r="J27">
         <v>174</v>
       </c>
+      <c r="K27">
+        <v>193</v>
+      </c>
       <c r="L27">
         <v>214</v>
       </c>
@@ -1510,6 +1566,9 @@
       <c r="P27">
         <v>173</v>
       </c>
+      <c r="Q27">
+        <v>123</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1545,6 +1604,9 @@
       <c r="P28">
         <v>19</v>
       </c>
+      <c r="Q28">
+        <v>3</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1601,6 +1663,9 @@
       <c r="P29">
         <v>0</v>
       </c>
+      <c r="Q29">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1618,6 +1683,9 @@
           <t>ESE HOSPITAL UNIVERSITARIO SAN JORGE DE PEREIRA</t>
         </is>
       </c>
+      <c r="D30">
+        <v>34</v>
+      </c>
       <c r="E30">
         <v>29</v>
       </c>
@@ -1710,6 +1778,9 @@
       <c r="P31">
         <v>0</v>
       </c>
+      <c r="Q31">
+        <v>1</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1766,6 +1837,9 @@
       <c r="P32">
         <v>54</v>
       </c>
+      <c r="Q32">
+        <v>56</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1819,6 +1893,9 @@
       <c r="P33">
         <v>18</v>
       </c>
+      <c r="Q33">
+        <v>11</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1872,6 +1949,9 @@
       <c r="P34">
         <v>9</v>
       </c>
+      <c r="Q34">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1890,7 +1970,7 @@
         </is>
       </c>
       <c r="D35">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="E35">
         <v>78</v>
@@ -1919,11 +1999,17 @@
       <c r="M35">
         <v>51</v>
       </c>
+      <c r="N35">
+        <v>55</v>
+      </c>
       <c r="O35">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="P35">
-        <v>45</v>
+        <v>40</v>
+      </c>
+      <c r="Q35">
+        <v>38</v>
       </c>
     </row>
     <row r="36">
@@ -1980,6 +2066,9 @@
       <c r="P37">
         <v>2</v>
       </c>
+      <c r="Q37">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2068,6 +2157,9 @@
       <c r="P39">
         <v>48</v>
       </c>
+      <c r="Q39">
+        <v>68</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2124,6 +2216,9 @@
       <c r="P40">
         <v>44</v>
       </c>
+      <c r="Q40">
+        <v>54</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2180,6 +2275,9 @@
       <c r="P41">
         <v>18</v>
       </c>
+      <c r="Q41">
+        <v>17</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2292,6 +2390,9 @@
       <c r="P43">
         <v>30</v>
       </c>
+      <c r="Q43">
+        <v>39</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2348,6 +2449,9 @@
       <c r="P44">
         <v>115</v>
       </c>
+      <c r="Q44">
+        <v>124</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2404,6 +2508,9 @@
       <c r="P45">
         <v>5</v>
       </c>
+      <c r="Q45">
+        <v>1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2460,6 +2567,9 @@
       <c r="P46">
         <v>95</v>
       </c>
+      <c r="Q46">
+        <v>69</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2478,7 +2588,7 @@
         </is>
       </c>
       <c r="D47">
-        <v>0</v>
+        <v>41</v>
       </c>
       <c r="J47">
         <v>15</v>
@@ -2501,6 +2611,9 @@
       <c r="P47">
         <v>39</v>
       </c>
+      <c r="Q47">
+        <v>58</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2557,6 +2670,9 @@
       <c r="P48">
         <v>1</v>
       </c>
+      <c r="Q48">
+        <v>4</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2613,6 +2729,9 @@
       <c r="P49">
         <v>0</v>
       </c>
+      <c r="Q49">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2666,6 +2785,9 @@
       <c r="P50">
         <v>2</v>
       </c>
+      <c r="Q50">
+        <v>3</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2775,6 +2897,9 @@
       <c r="P52">
         <v>1</v>
       </c>
+      <c r="Q52">
+        <v>5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2831,6 +2956,9 @@
       <c r="P53">
         <v>0</v>
       </c>
+      <c r="Q53">
+        <v>4</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2887,6 +3015,9 @@
       <c r="P54">
         <v>0</v>
       </c>
+      <c r="Q54">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2943,6 +3074,9 @@
       <c r="P55">
         <v>10</v>
       </c>
+      <c r="Q55">
+        <v>18</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2960,6 +3094,9 @@
           <t>SANIDAD POLICIA NACIONAL RISARALDA</t>
         </is>
       </c>
+      <c r="D56">
+        <v>31</v>
+      </c>
       <c r="E56">
         <v>10</v>
       </c>
@@ -2996,6 +3133,9 @@
       <c r="P56">
         <v>40</v>
       </c>
+      <c r="Q56">
+        <v>18</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3048,6 +3188,9 @@
       </c>
       <c r="P57">
         <v>26</v>
+      </c>
+      <c r="Q57">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>